<commit_message>
Bug fixes and hair color potion revisions.
</commit_message>
<xml_diff>
--- a/Economy.xlsx
+++ b/Economy.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="19001"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\The Dungeon\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dungeon_depths\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Item Name</t>
   </si>
@@ -213,6 +213,18 @@
   </si>
   <si>
     <t>Masculine Potion</t>
+  </si>
+  <si>
+    <t>Breast Shrinking Potion</t>
+  </si>
+  <si>
+    <t>Hyperheal Potion</t>
+  </si>
+  <si>
+    <t>Hypermana Potion</t>
+  </si>
+  <si>
+    <t>Spidersilk Whip</t>
   </si>
 </sst>
 </file>
@@ -293,7 +305,34 @@
     </cx:data>
   </cx:chartData>
   <cx:chart>
-    <cx:title pos="t" align="ctr" overlay="0"/>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Price Distribution </cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Price Distribution </a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
         <cx:series layoutId="clusteredColumn" uniqueId="{2F54256D-AD04-40C5-9C11-150F796D8A2B}">
@@ -1245,10 +1284,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{958984CE-5666-4795-868B-A9D0A5A5C02F}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1739,6 +1778,38 @@
         <v>300</v>
       </c>
     </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>64</v>
+      </c>
+      <c r="B64">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>65</v>
+      </c>
+      <c r="B65">
+        <v>900</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>